<commit_message>
chore: actualizar plantilla de incidencias
</commit_message>
<xml_diff>
--- a/backend/incidencias.xlsx
+++ b/backend/incidencias.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C82A1926-111B-405A-AC3A-A9B9015E4864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>REPORTE DE ASISTENCIA E INCIDENCIAS - HOSANNA INFANTIL</t>
   </si>
@@ -22,9 +36,6 @@
     <t>Localidad:</t>
   </si>
   <si>
-    <t>Fecha:</t>
-  </si>
-  <si>
     <t>REPORTE DE ASISTENCIA</t>
   </si>
   <si>
@@ -86,12 +97,18 @@
   </si>
   <si>
     <t>Observaciones Generales</t>
+  </si>
+  <si>
+    <t>Linda Vista</t>
+  </si>
+  <si>
+    <t>Fecha: 12/7/2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -246,60 +263,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -319,9 +335,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -359,9 +375,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -396,7 +412,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -431,7 +447,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -604,301 +620,351 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" customWidth="1"/>
-    <col min="2" max="5" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="16.26953125" customWidth="1"/>
+    <col min="2" max="3" width="13.7265625" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" spans="1:5" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="12"/>
+    </row>
+    <row r="2" spans="1:5" ht="6.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="17"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="18"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="8"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="12"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="12"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="14" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="B8" s="6">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6">
+        <v>2</v>
+      </c>
+      <c r="E8" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15">
-        <f>SUM(B8:D8)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="B9" s="6">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6">
+        <v>2</v>
+      </c>
+      <c r="E9" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15">
-        <f t="shared" ref="E9:E17" si="0">SUM(B9:D9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="B10" s="6">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6">
+        <v>4</v>
+      </c>
+      <c r="D10" s="6">
+        <v>4</v>
+      </c>
+      <c r="E10" s="6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="B11" s="6">
+        <v>2</v>
+      </c>
+      <c r="C11" s="6">
+        <v>7</v>
+      </c>
+      <c r="D11" s="6">
+        <v>5</v>
+      </c>
+      <c r="E11" s="6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="B12" s="6">
+        <v>3</v>
+      </c>
+      <c r="C12" s="6">
+        <v>5</v>
+      </c>
+      <c r="D12" s="6">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="B13" s="6">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6">
+        <v>10</v>
+      </c>
+      <c r="D13" s="6">
+        <v>2</v>
+      </c>
+      <c r="E13" s="6">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="B14" s="6">
+        <v>8</v>
+      </c>
+      <c r="C14" s="6">
+        <v>7</v>
+      </c>
+      <c r="D14" s="6">
+        <v>5</v>
+      </c>
+      <c r="E14" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="B15" s="6">
+        <v>8</v>
+      </c>
+      <c r="C15" s="6">
+        <v>3</v>
+      </c>
+      <c r="D15" s="6">
+        <v>4</v>
+      </c>
+      <c r="E15" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="B16" s="6">
+        <v>3</v>
+      </c>
+      <c r="C16" s="6">
+        <v>6</v>
+      </c>
+      <c r="D16" s="6">
+        <v>2</v>
+      </c>
+      <c r="E16" s="6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="6">
+        <v>38</v>
+      </c>
+      <c r="C17" s="6">
+        <v>46</v>
+      </c>
+      <c r="D17" s="6">
+        <v>27</v>
+      </c>
+      <c r="E17" s="6">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="15">
-        <f>SUM(B8:B16)</f>
-        <v>0</v>
-      </c>
-      <c r="C17" s="15">
-        <f t="shared" ref="C17:D17" si="1">SUM(C8:C16)</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E17" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+      <c r="B19">
+        <v>12</v>
+      </c>
+      <c r="C19">
+        <v>11</v>
+      </c>
+      <c r="D19">
+        <v>10</v>
+      </c>
+      <c r="E19">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16">
-        <f>SUM(B19:D19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" spans="1:5" ht="85" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-    </row>
-    <row r="22" spans="1:5" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="1:5" ht="85" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-    </row>
-    <row r="23" spans="1:5" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="18" t="s">
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="1:5" ht="85" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-    </row>
-    <row r="24" spans="1:5" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="1:5" ht="85" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-    </row>
-    <row r="26" spans="1:5" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A6:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>